<commit_message>
template uploaded new one
</commit_message>
<xml_diff>
--- a/public/templates/vendor_upload_template.xlsx
+++ b/public/templates/vendor_upload_template.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\timesheet-app\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F039B800-EE24-4F3A-86A2-ADBC6810A419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2B0DB938-8532-4744-B2FE-2E5516201F27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{013FBE18-F61B-431E-9C57-53EF7E3B5338}"/>
   </bookViews>
   <sheets>
     <sheet name="Vendor" sheetId="1" r:id="rId1"/>
-    <sheet name="data" sheetId="3" state="hidden" r:id="rId2"/>
+    <sheet name="data" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
   <si>
     <t>Email</t>
   </si>
@@ -72,30 +72,18 @@
     <t>SubTeams</t>
   </si>
   <si>
-    <t>BA</t>
-  </si>
-  <si>
     <t>QA</t>
   </si>
   <si>
     <t>DEV</t>
   </si>
   <si>
-    <t>DBA</t>
-  </si>
-  <si>
-    <t>PMO</t>
-  </si>
-  <si>
     <t>Optime-Tech</t>
   </si>
   <si>
     <t>Yovant</t>
   </si>
   <si>
-    <t>ScrumMaster</t>
-  </si>
-  <si>
     <t>LTM</t>
   </si>
   <si>
@@ -108,13 +96,61 @@
     <t>EY</t>
   </si>
   <si>
-    <t>DuckCreek</t>
-  </si>
-  <si>
     <t>NTT Data</t>
   </si>
   <si>
     <t>Invenger</t>
+  </si>
+  <si>
+    <t>Data Engineer</t>
+  </si>
+  <si>
+    <t>DTC</t>
+  </si>
+  <si>
+    <t>MySlide</t>
+  </si>
+  <si>
+    <t>Websites</t>
+  </si>
+  <si>
+    <t>Integrations</t>
+  </si>
+  <si>
+    <t>PolicyAttach</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>IT GRC</t>
+  </si>
+  <si>
+    <t>IT Ops</t>
+  </si>
+  <si>
+    <t>Delivery/Scrum Master</t>
+  </si>
+  <si>
+    <t>BSA</t>
+  </si>
+  <si>
+    <t>Release Management</t>
+  </si>
+  <si>
+    <t>Analyst</t>
+  </si>
+  <si>
+    <t>EITACIES</t>
+  </si>
+  <si>
+    <t>Exavalu</t>
+  </si>
+  <si>
+    <t>NEST</t>
   </si>
 </sst>
 </file>
@@ -521,21 +557,21 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2FB9D2DC-88F9-4B2D-8B07-2AD0A5941689}">
           <x14:formula1>
-            <xm:f>data!$C$2:$C$14</xm:f>
+            <xm:f>data!$C$2:$C$20</xm:f>
           </x14:formula1>
           <xm:sqref>E2:E1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0FA41776-A8B2-41D4-962D-58E40DD6F8EB}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A337F88A-649D-4D4A-B1A4-B345B60A9A35}">
           <x14:formula1>
-            <xm:f>data!$A$2:$A$5</xm:f>
+            <xm:f>data!$B$2:$B$15</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2:D1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E4E6CD72-44CA-4FF2-8BE5-60B327E81574}">
+          <x14:formula1>
+            <xm:f>data!$A$2:$A$24</xm:f>
           </x14:formula1>
           <xm:sqref>C2:C1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A337F88A-649D-4D4A-B1A4-B345B60A9A35}">
-          <x14:formula1>
-            <xm:f>data!$B$2:$B$7</xm:f>
-          </x14:formula1>
-          <xm:sqref>D2:D1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -545,16 +581,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43AA28A4-1708-49C1-9939-94064891E6E1}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.21875" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -565,150 +600,126 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2" t="str">
-        <f>"'"&amp;B2&amp;"'),"</f>
-        <v>'PMO'),</v>
-      </c>
-      <c r="I2" t="str">
-        <f>"("&amp;G2&amp;","&amp;H2</f>
-        <v>(4,'PMO'),</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
       <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3">
-        <v>4</v>
-      </c>
-      <c r="H3" t="str">
-        <f t="shared" ref="H3:H7" si="0">"'"&amp;B3&amp;"'),"</f>
-        <v>'DEV'),</v>
-      </c>
-      <c r="I3" t="str">
-        <f t="shared" ref="I3:I7" si="1">"("&amp;G3&amp;","&amp;H3</f>
-        <v>(4,'DEV'),</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4">
-        <v>4</v>
-      </c>
-      <c r="H4" t="str">
-        <f t="shared" si="0"/>
-        <v>'QA'),</v>
-      </c>
-      <c r="I4" t="str">
-        <f t="shared" si="1"/>
-        <v>(4,'QA'),</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s">
         <v>19</v>
       </c>
-      <c r="G5">
-        <v>4</v>
-      </c>
-      <c r="H5" t="str">
-        <f t="shared" si="0"/>
-        <v>'BA'),</v>
-      </c>
-      <c r="I5" t="str">
-        <f t="shared" si="1"/>
-        <v>(4,'BA'),</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
         <v>20</v>
       </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-      <c r="H6" t="str">
-        <f t="shared" si="0"/>
-        <v>'DBA'),</v>
-      </c>
-      <c r="I6" t="str">
-        <f t="shared" si="1"/>
-        <v>(4,'DBA'),</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G7">
-        <v>4</v>
-      </c>
-      <c r="H7" t="str">
-        <f t="shared" si="0"/>
-        <v>'ScrumMaster'),</v>
-      </c>
-      <c r="I7" t="str">
-        <f t="shared" si="1"/>
-        <v>(4,'ScrumMaster'),</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="C8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="C9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="C10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="C11" t="s">
-        <v>25</v>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>